<commit_message>
DOE v3: add Phase 0 isolating acquisition-skip penalty; downgrade px-vs-match claim
Operators skip acquisition and reuse stale recipes in production, so merged
match rates confound kV, pixel count, and CAD freshness. v3 adds P1/P2/P3
(same wafer, same inspection params, fresh vs reused CAD), makes the R sweep a
controlled px-vs-match experiment (adds R=2.0 point), and keeps kV/N/Frame/tact
phases. Run sheet gains a Phase0 sheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AEDPo1aa2m4Ui6JuqiXEbY
</commit_message>
<xml_diff>
--- a/Xray_DOE_RunSheet.xlsx
+++ b/Xray_DOE_RunSheet.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhaseA_kV확정" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhaseB_N곡선_Frame" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhaseC_검증" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="분석_자동계산" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase0_취득페널티" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhaseA_kV확정" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhaseB_N곡선_Frame" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhaseC_검증" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="분석_자동계산" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,6 +469,275 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Phase0 — 취득 생략 페널티 분리 (최우선: 같은 웨이퍼, CAD 신선도만 변경)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>검사 파라미터는 P1·P2 완전 동일. P2−P1 매칭률 차이 = 취득 생략 페널티</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>자재</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>CAD 신선도</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>kV</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Frame</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>측정직경(µm)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>nominal(µm)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Q_dia(자동)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>매칭 성공die</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>검사die수</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>void%</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>tact(초)</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>판정(자동)</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>메모</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>182µm</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>기존 레시피(취득 생략=현행)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="4" t="n">
+        <v>182</v>
+      </c>
+      <c r="I5" s="6">
+        <f>IFERROR(G5/H5,"")</f>
+        <v/>
+      </c>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L5" s="5" t="n"/>
+      <c r="M5" s="5" t="n"/>
+      <c r="N5" s="7">
+        <f>IF(J5="","",J5&amp;"/"&amp;K5&amp;" 매칭")</f>
+        <v/>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>현행 운용 기준선</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>182µm</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>신규 취득 후 검사</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="4" t="n">
+        <v>182</v>
+      </c>
+      <c r="I6" s="6">
+        <f>IFERROR(G6/H6,"")</f>
+        <v/>
+      </c>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="7">
+        <f>IF(J6="","",J6&amp;"/"&amp;K6&amp;" 매칭")</f>
+        <v/>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>P1과 매칭률 비교</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>TB500M</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>기존 RUN 레시피 재사용</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="I7" s="6">
+        <f>IFERROR(G7/H7,"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="7">
+        <f>IF(J7="","",J7&amp;"/"&amp;K7&amp;" 매칭")</f>
+        <v/>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>PhaseB 신규취득 결과와 비교</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -756,13 +1026,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1189,12 +1459,52 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>B4b</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>TB500M</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>B0 kV</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
+      <c r="J12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K12" s="4" t="n"/>
+      <c r="L12" s="4" t="n"/>
+      <c r="M12" s="4" t="n"/>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>26px 아래 두번째 점(13px) — 취득R 상한 검증</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1406,7 +1716,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add PhaseW power-sweep sheet to run sheet; cross-reference W correction
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AEDPo1aa2m4Ui6JuqiXEbY
</commit_message>
<xml_diff>
--- a/Xray_DOE_RunSheet.xlsx
+++ b/Xray_DOE_RunSheet.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhaseB_N곡선_Frame" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhaseC_검증" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="분석_자동계산" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhaseW_Power" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1823,4 +1824,439 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PhaseW — Power 스윕 (158µm 전용, 26µm는 4W 고정)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>고정: kV*(PhaseA 결과), R(모델값), F32, 같은 die·AOI·범프 추적 | 판정: 깜빡임void 수·void%σ·수렴 + 가드(경계폭·Q_dia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>반복#</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>측정직경(µm)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>nominal(µm)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Q_dia(자동)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>매칭die</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>검사die</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>void%</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>깜빡임void수</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>경계폭(px)</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>tact(초)</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>메모</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="G5" s="6">
+        <f>IFERROR(E5/F5,"")</f>
+        <v/>
+      </c>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
+      <c r="M5" s="5" t="n"/>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>기준점</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="G6" s="6">
+        <f>IFERROR(E6/F6,"")</f>
+        <v/>
+      </c>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="G7" s="6">
+        <f>IFERROR(E7/F7,"")</f>
+        <v/>
+      </c>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="G8" s="6">
+        <f>IFERROR(E8/F8,"")</f>
+        <v/>
+      </c>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
+      <c r="L8" s="5" t="n"/>
+      <c r="M8" s="5" t="n"/>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>저측(악화방향 확인)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="G9" s="6">
+        <f>IFERROR(E9/F9,"")</f>
+        <v/>
+      </c>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" s="5" t="n"/>
+      <c r="K9" s="5" t="n"/>
+      <c r="L9" s="5" t="n"/>
+      <c r="M9" s="5" t="n"/>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>중간점</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="G10" s="6">
+        <f>IFERROR(E10/F10,"")</f>
+        <v/>
+      </c>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
+      <c r="L10" s="5" t="n"/>
+      <c r="M10" s="5" t="n"/>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>고측+블러가드</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="G11" s="6">
+        <f>IFERROR(E11/F11,"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J11" s="5" t="n"/>
+      <c r="K11" s="5" t="n"/>
+      <c r="L11" s="5" t="n"/>
+      <c r="M11" s="5" t="n"/>
+      <c r="N11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="G12" s="6">
+        <f>IFERROR(E12/F12,"")</f>
+        <v/>
+      </c>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="5" t="n"/>
+      <c r="L12" s="5" t="n"/>
+      <c r="M12" s="5" t="n"/>
+      <c r="N12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>8(허용시)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="G13" s="6">
+        <f>IFERROR(E13/F13,"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
+      <c r="L13" s="5" t="n"/>
+      <c r="M13" s="5" t="n"/>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>W·F 교환검증: (4W,F32)와 void% 비교</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>